<commit_message>
Update QuizTok app with latest changes and new files
</commit_message>
<xml_diff>
--- a/data/quizzes.xlsx
+++ b/data/quizzes.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="quizzes" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="questions" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="quizzes" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="questions" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -668,6 +668,166 @@
       <c r="H6" t="inlineStr">
         <is>
           <t>2026-07-03 10:56:49</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>bank-260703-140125</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Banking Ops Battle</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>🏦</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>IVR</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>20</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>admin@citi.com</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>2026-07-03 14:01:25</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>bank-260703-140439</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Banking Ops Battle - IVR</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>🏦</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>IVR</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>20</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>admin@citi.com</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>2026-07-03 14:04:39</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>bank-260703-141304</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>IVR</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>🏦</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>IVR</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>20</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>admin@citi.com</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>2026-07-03 14:13:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>bank-260703-143043</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Banking Ops Battle</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>🏦</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>KPI &amp; Metrics + IVR</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>20</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>admin@citi.com</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>2026-07-03 14:30:43</t>
         </is>
       </c>
     </row>
@@ -682,7 +842,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K32"/>
+  <dimension ref="A1:K67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2255,6 +2415,1731 @@
         <v>1000</v>
       </c>
     </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>bank-260703-140125</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>0</v>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>subjective</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>How would you explain 'why KYC matters' to an annoyed customer in one breath?</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr"/>
+      <c r="F33" t="inlineStr"/>
+      <c r="G33" t="inlineStr"/>
+      <c r="H33" t="inlineStr"/>
+      <c r="I33" t="inlineStr"/>
+      <c r="J33" t="n">
+        <v>45</v>
+      </c>
+      <c r="K33" t="n">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>bank-260703-140125</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>1</v>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>mcq</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>The IVR handled 4700 calls; 3260 completed without reaching an agent. Containment rate = ?</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>69.4%</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>81.9%</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>72.4%</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>64.4%</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="J34" t="n">
+        <v>30</v>
+      </c>
+      <c r="K34" t="n">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>bank-260703-140125</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>2</v>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>mcq</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>The IVR handled 3200 calls; 1711 completed without reaching an agent. Containment rate = ?</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>53.5%</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>45.5%</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>62%</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>56.5%</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="J35" t="n">
+        <v>30</v>
+      </c>
+      <c r="K35" t="n">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>bank-260703-140125</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>3</v>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>mcq</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>The IVR handled 2800 calls; 1810 completed without reaching an agent. Containment rate = ?</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>64.6%</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>70.1%</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>69.6%</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>72.6%</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="J36" t="n">
+        <v>30</v>
+      </c>
+      <c r="K36" t="n">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>bank-260703-140125</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>4</v>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>mcq</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>The IVR handled 4500 calls; 2743 completed without reaching an agent. Containment rate = ?</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>66%</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>69.5%</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>76%</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>61%</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="J37" t="n">
+        <v>30</v>
+      </c>
+      <c r="K37" t="n">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>bank-260703-140125</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>5</v>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>mcq</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>The IVR handled 1900 calls; 1139 completed without reaching an agent. Containment rate = ?</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>63.4%</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>72.4%</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>56.9%</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>59.9%</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="J38" t="n">
+        <v>30</v>
+      </c>
+      <c r="K38" t="n">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>bank-260703-140125</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>6</v>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>mcq</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>The IVR handled 1900 calls; 1410 completed without reaching an agent. Containment rate = ?</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>82.2%</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>77.7%</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>62.2%</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>74.2%</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="J39" t="n">
+        <v>30</v>
+      </c>
+      <c r="K39" t="n">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>bank-260703-140125</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>7</v>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>mcq</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>The IVR handled 2700 calls; 2126 completed without reaching an agent. Containment rate = ?</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>78.7%</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>76.2%</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>82.2%</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>94.2%</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="J40" t="n">
+        <v>30</v>
+      </c>
+      <c r="K40" t="n">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>bank-260703-140125</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>8</v>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>mcq</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>What does DNIS stand for?</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Dialed Number Identification Service</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Barge-In</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>Text To Speech</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>Voice User Interface</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="J41" t="n">
+        <v>20</v>
+      </c>
+      <c r="K41" t="n">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>bank-260703-140125</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>9</v>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>mcq</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Which statement about TTS is TRUE?</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>TTS means: converting text into spoken audio prompts</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>TTS means: share of callers pressing to leave the IVR for an agent</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>TTS means: identifying which number the caller dialled</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>TTS means: customer record opening automatically as the call arrives</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="J42" t="n">
+        <v>20</v>
+      </c>
+      <c r="K42" t="n">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>bank-260703-140439</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>0</v>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>subjective</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>A VIP customer got wrong information yesterday. Draft your callback opening line.</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr"/>
+      <c r="F43" t="inlineStr"/>
+      <c r="G43" t="inlineStr"/>
+      <c r="H43" t="inlineStr"/>
+      <c r="I43" t="inlineStr"/>
+      <c r="J43" t="n">
+        <v>45</v>
+      </c>
+      <c r="K43" t="n">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>bank-260703-140439</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>1</v>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>mcq</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>What does IVR stand for?</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Interactive Voice Response</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Natural Language Understanding (IVR)</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>Barge-In</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>Menu Depth</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="J44" t="n">
+        <v>20</v>
+      </c>
+      <c r="K44" t="n">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>bank-260703-140439</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>2</v>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>mcq</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>What does SPOP stand for?</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Skill Based Routing</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Automatic Number Identification</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>Dialed Number Identification Service</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>Screen Pop</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="J45" t="n">
+        <v>20</v>
+      </c>
+      <c r="K45" t="n">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>bank-260703-140439</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>3</v>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>mcq</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Barge-in in an IVR means:</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Callers can respond before the prompt finishes</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>IVR hanging up on silence</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>Supervisors joining calls</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>Agents interrupting customers</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="J46" t="n">
+        <v>25</v>
+      </c>
+      <c r="K46" t="n">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>bank-260703-140439</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>4</v>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>mcq</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Which term matches this definition: “extracting caller intent from free speech instead of menus”?</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>NLUI (Natural Language Understanding (IVR))</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>TTS (Text To Speech)</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>CCB (Courtesy Callback)</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>SBR (Skill Based Routing)</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="J47" t="n">
+        <v>20</v>
+      </c>
+      <c r="K47" t="n">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>bank-260703-140439</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>5</v>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>mcq</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>What does ANI stand for?</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Automatic Number Identification</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>Barge-In</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>Opt-Out Rate</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>Courtesy Callback</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="J48" t="n">
+        <v>20</v>
+      </c>
+      <c r="K48" t="n">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>bank-260703-140439</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>6</v>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>mcq</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Which term matches this definition: “caller's phone number captured automatically”?</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>IVR (Interactive Voice Response)</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>VUI (Voice User Interface)</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>ANI (Automatic Number Identification)</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>SPOP (Screen Pop)</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="J49" t="n">
+        <v>20</v>
+      </c>
+      <c r="K49" t="n">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>bank-260703-140439</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>7</v>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>mcq</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Which term matches this definition: “share of callers pressing to leave the IVR for an agent”?</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>DTMF (Dual Tone Multi Frequency)</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>SBR (Skill Based Routing)</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>OPTR (Opt-Out Rate)</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>IVR (Interactive Voice Response)</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="J50" t="n">
+        <v>20</v>
+      </c>
+      <c r="K50" t="n">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>bank-260703-140439</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>8</v>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>mcq</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>What does TTS stand for?</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Voice User Interface</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>Skill Based Routing</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>Automatic Call Distributor</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>Text To Speech</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="J51" t="n">
+        <v>20</v>
+      </c>
+      <c r="K51" t="n">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>bank-260703-140439</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>9</v>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>mcq</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Which term matches this definition: “customer record opening automatically as the call arrives”?</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>SPOP (Screen Pop)</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>ASR (Automatic Speech Recognition)</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>MDEP (Menu Depth)</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>DTMF (Dual Tone Multi Frequency)</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="J52" t="n">
+        <v>20</v>
+      </c>
+      <c r="K52" t="n">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>bank-260703-141304</t>
+        </is>
+      </c>
+      <c r="B53" t="n">
+        <v>0</v>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>mcq</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>What does VUI stand for?</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Dual Tone Multi Frequency</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>Voice User Interface</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>Courtesy Callback</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>Skill Based Routing</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="J53" t="n">
+        <v>20</v>
+      </c>
+      <c r="K53" t="n">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>bank-260703-141304</t>
+        </is>
+      </c>
+      <c r="B54" t="n">
+        <v>1</v>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>subjective</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>An elderly customer struggles with the mobile app. How would you help without pushing them away from digital?</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr"/>
+      <c r="F54" t="inlineStr"/>
+      <c r="G54" t="inlineStr"/>
+      <c r="H54" t="inlineStr"/>
+      <c r="I54" t="inlineStr"/>
+      <c r="J54" t="n">
+        <v>45</v>
+      </c>
+      <c r="K54" t="n">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>bank-260703-141304</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
+        <v>2</v>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>mcq</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Which term matches this definition: “caller's phone number captured automatically”?</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>IVR (Interactive Voice Response)</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>VUI (Voice User Interface)</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>ANI (Automatic Number Identification)</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>SPOP (Screen Pop)</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="J55" t="n">
+        <v>20</v>
+      </c>
+      <c r="K55" t="n">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>bank-260703-141304</t>
+        </is>
+      </c>
+      <c r="B56" t="n">
+        <v>3</v>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>mcq</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>A caller says 'I lost my debit card' to the open-ended IVR prompt. Which technology maps this to the card-block flow?</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>DTMF</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>Text To Speech</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>Screen pop</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>Natural Language Understanding</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="J56" t="n">
+        <v>25</v>
+      </c>
+      <c r="K56" t="n">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>bank-260703-141304</t>
+        </is>
+      </c>
+      <c r="B57" t="n">
+        <v>4</v>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>mcq</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>What does OPTR stand for?</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Voice User Interface</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>Courtesy Callback</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>Menu Depth</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>Opt-Out Rate</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="J57" t="n">
+        <v>20</v>
+      </c>
+      <c r="K57" t="n">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>bank-260703-143043</t>
+        </is>
+      </c>
+      <c r="B58" t="n">
+        <v>0</v>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>mcq</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>An agent handled 40 calls with total talk 7240s, hold 1400s and ACW 1240s. AHT in seconds = ?</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>232 sec</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>217 sec</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>307 sec</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>247 sec</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="J58" t="n">
+        <v>30</v>
+      </c>
+      <c r="K58" t="n">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>bank-260703-143043</t>
+        </is>
+      </c>
+      <c r="B59" t="n">
+        <v>1</v>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>mcq</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>2500 calls were offered and 345 callers hung up before answer. What is the abandonment rate?</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>28.8%</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>10.8%</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>17.3%</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>13.8%</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="J59" t="n">
+        <v>30</v>
+      </c>
+      <c r="K59" t="n">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>bank-260703-143043</t>
+        </is>
+      </c>
+      <c r="B60" t="n">
+        <v>2</v>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>mcq</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>1400 calls were offered and 60 callers hung up before answer. What is the abandonment rate?</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>1.3%</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>12.8%</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>9.8%</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>4.3%</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="J60" t="n">
+        <v>30</v>
+      </c>
+      <c r="K60" t="n">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>bank-260703-143043</t>
+        </is>
+      </c>
+      <c r="B61" t="n">
+        <v>3</v>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>mcq</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>600 calls were offered and 43 callers hung up before answer. What is the abandonment rate?</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>4.7%</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>7.2%</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>2.7%</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>19.2%</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="J61" t="n">
+        <v>30</v>
+      </c>
+      <c r="K61" t="n">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>bank-260703-143043</t>
+        </is>
+      </c>
+      <c r="B62" t="n">
+        <v>4</v>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>mcq</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>The IVR handled 1700 calls; 664 completed without reaching an agent. Containment rate = ?</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>44.1%</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>36.6%</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>39.1%</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>42.1%</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="J62" t="n">
+        <v>30</v>
+      </c>
+      <c r="K62" t="n">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>bank-260703-143043</t>
+        </is>
+      </c>
+      <c r="B63" t="n">
+        <v>5</v>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>mcq</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>What does NLUI stand for?</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>Screen Pop</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>Skill Based Routing</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>Natural Language Understanding (IVR)</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>Dialed Number Identification Service</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="J63" t="n">
+        <v>20</v>
+      </c>
+      <c r="K63" t="n">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>bank-260703-143043</t>
+        </is>
+      </c>
+      <c r="B64" t="n">
+        <v>6</v>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>mcq</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>900 calls were offered and 62 callers hung up before answer. What is the abandonment rate?</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>11.9%</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>3.9%</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>15.4%</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>6.9%</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="J64" t="n">
+        <v>30</v>
+      </c>
+      <c r="K64" t="n">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>bank-260703-143043</t>
+        </is>
+      </c>
+      <c r="B65" t="n">
+        <v>7</v>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>mcq</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>An agent was scheduled 144 hours this month; 36 hours went to leave, training and breaks. Shrinkage = ?</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>13.5%</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>33%</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="J65" t="n">
+        <v>30</v>
+      </c>
+      <c r="K65" t="n">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>bank-260703-143043</t>
+        </is>
+      </c>
+      <c r="B66" t="n">
+        <v>8</v>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>mcq</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>In an NPS survey, 56% were promoters, 5% detractors and the rest passives. NPS = ?</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>56</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>51</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>41</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>46</t>
+        </is>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="J66" t="n">
+        <v>30</v>
+      </c>
+      <c r="K66" t="n">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>bank-260703-143043</t>
+        </is>
+      </c>
+      <c r="B67" t="n">
+        <v>9</v>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>mcq</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>What does ANI stand for?</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>Automatic Number Identification</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>Barge-In</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>Opt-Out Rate</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>Courtesy Callback</t>
+        </is>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="J67" t="n">
+        <v>20</v>
+      </c>
+      <c r="K67" t="n">
+        <v>1000</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>